<commit_message>
Update employee directory with corrected numbers
- Fill in Kenzie (502) 650-2273 and Nathan (502) 693-8371
- Reinstate Lidy (corrected to 502-381-0680) and Madison as Active
- Remove the other crossed-out entry
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,12 +32,8 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00777777"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -48,12 +44,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C8102E"/>
         <bgColor rgb="00C8102E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,15 +73,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -459,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -696,24 +683,24 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(502) 650-????</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Active — number partially obscured</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -725,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Madison</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 438-7200</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -742,29 +729,29 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 603-????</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Active — number partially obscured</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0655</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -776,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -793,73 +780,56 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>(270) 874-0655</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Samuel</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>(502) 724-2384</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>Vicki</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>(502) 701-9597</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Grace</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>(316) 391-8735</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Crossed out on list</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Lidy</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>(502) 381-0180</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Crossed out on list</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Madison</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>(502) 438-7200</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Crossed out on list</t>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C23"/>
+  <autoFilter ref="A1:C22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(directory): remove Madison (crossed-out), regenerate xlsx+pdf — 20 active
Bobby's corrections 2026-04-26:
- Madison removed (was on the crossed-out list)
- Kenzie/Nathan/Lidy already correct from prior session
- Spec doc: Employee List + Phone Directory rows flipped 🟢

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -712,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Madison</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(502) 438-7200</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Richard</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(270) 874-0655</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0655</t>
+          <t>(502) 724-2384</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Vicki</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(502) 701-9597</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -811,25 +811,8 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Vicki</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>(502) 701-9597</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C22"/>
+  <autoFilter ref="A1:C21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Zach + Dakayla to employee directory (20 -> 22 active)
Two new hires Bobby onboarded last week. Phone numbers extracted from
background-check forms. Regenerated employee_directory.xlsx + .pdf.

Going forward, the outlook-daily-pull-7am skill will surface a 'New Hires'
section above Director's Corner with name, phone, hiring stage, and the
proposed one-line directory edit, so onboarding never gets buried again.
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -542,12 +542,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Divan</t>
+          <t>Dakayla</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-9406</t>
+          <t>(502) 537-8724</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -559,12 +559,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Divan</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>(407) 456-1445</t>
+          <t>(502) 821-9406</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -576,12 +576,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>(502) 527-1477</t>
+          <t>(407) 456-1445</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -593,12 +593,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Jada</t>
+          <t>Grace</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-5962</t>
+          <t>(502) 527-1477</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -610,12 +610,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Jeremiah</t>
+          <t>Jada</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>(502) 498-9401</t>
+          <t>(502) 821-5962</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -627,12 +627,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Jeremiah</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>(502) 606-3088</t>
+          <t>(502) 498-9401</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -644,12 +644,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Kasey</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>(502) 884-2273</t>
+          <t>(502) 606-3088</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kasey</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>(502) 531-8704</t>
+          <t>(502) 884-2273</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -678,12 +678,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(502) 650-2273</t>
+          <t>(502) 531-8704</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -695,12 +695,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(502) 381-0680</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -712,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0655</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Richard</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(270) 874-0655</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,22 +797,56 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>Samuel</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>(502) 724-2384</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>Vicki</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>(502) 701-9597</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Zach</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>(502) 422-9066</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C21"/>
+  <autoFilter ref="A1:C23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
directory: add Nyatiek (new hire 2026-05-05, phone pending)
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Employees" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Nyatiek</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0655</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Richard</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(270) 874-0655</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Vicki</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(502) 701-9597</t>
+          <t>(502) 724-2384</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -831,22 +831,39 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>(502) 701-9597</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>Zach</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>(502) 422-9066</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C23"/>
+  <autoFilter ref="A1:C24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
directory: Richard → Richard Gibbs, phone 0655 → 0688 (correction)
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0655</t>
+          <t>(270) 874-0688</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">

</xml_diff>

<commit_message>
directory: add Anthony (new hire 2026-05-12) — phone pending
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Ash</t>
+          <t>Anthony</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>(502) 554-4833</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -508,12 +508,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Autumn</t>
+          <t>Ash</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>(502) 656-2133</t>
+          <t>(502) 554-4833</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -525,12 +525,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Bri</t>
+          <t>Autumn</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>(502) 202-4126</t>
+          <t>(502) 656-2133</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -542,12 +542,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Dakayla</t>
+          <t>Bri</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>(502) 537-8724</t>
+          <t>(502) 202-4126</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -559,12 +559,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Divan</t>
+          <t>Dakayla</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-9406</t>
+          <t>(502) 537-8724</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -576,12 +576,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Divan</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>(407) 456-1445</t>
+          <t>(502) 821-9406</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -593,12 +593,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>(502) 527-1477</t>
+          <t>(407) 456-1445</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -610,12 +610,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Jada</t>
+          <t>Grace</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-5962</t>
+          <t>(502) 527-1477</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -627,12 +627,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Jeremiah</t>
+          <t>Jada</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>(502) 498-9401</t>
+          <t>(502) 821-5962</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -644,12 +644,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Jeremiah</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>(502) 606-3088</t>
+          <t>(502) 498-9401</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Kasey</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>(502) 884-2273</t>
+          <t>(502) 606-3088</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -678,12 +678,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kasey</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(502) 531-8704</t>
+          <t>(502) 884-2273</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -695,12 +695,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(502) 650-2273</t>
+          <t>(502) 531-8704</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -712,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(502) 381-0680</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Nyatiek</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(502) 576-1634</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0688</t>
+          <t>(502) 576-1634</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(270) 874-0688</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Vicki</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(502) 701-9597</t>
+          <t>(502) 724-2384</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -848,22 +848,39 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>(502) 701-9597</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>Zach</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>(502) 422-9066</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C24"/>
+  <autoFilter ref="A1:C25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Daily brief 2026-06-12 — team notes + dashboard wire + new hires Ryan/Damon (rescue)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -576,12 +576,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Divan</t>
+          <t>Damon</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-9406</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -593,12 +593,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Divan</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>(407) 456-1445</t>
+          <t>(502) 821-9406</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -610,12 +610,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>(502) 527-1477</t>
+          <t>(407) 456-1445</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -627,12 +627,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Jada</t>
+          <t>Grace</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-5962</t>
+          <t>(502) 527-1477</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -644,12 +644,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Jeremiah</t>
+          <t>Jada</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>(502) 498-9401</t>
+          <t>(502) 821-5962</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Jeremiah</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>(502) 606-3088</t>
+          <t>(502) 498-9401</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -678,12 +678,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Kasey</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(502) 884-2273</t>
+          <t>(502) 606-3088</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -695,12 +695,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kasey</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(502) 531-8704</t>
+          <t>(502) 884-2273</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -712,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(502) 650-2273</t>
+          <t>(502) 531-8704</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 381-0680</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Nyatiek</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(502) 576-1634</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0688</t>
+          <t>(502) 576-1634</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(270) 874-0688</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -848,12 +848,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Vicki</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>(502) 701-9597</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -865,22 +865,56 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>Samuel</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>(502) 724-2384</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>(502) 701-9597</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>Zach</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>(502) 422-9066</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C25"/>
+  <autoFilter ref="A1:C27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
directory: add Angela (new hire 2026-06-16); refresh shop performance
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Anthony</t>
+          <t>Angela</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>(502) 938-5182</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -508,12 +508,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Ash</t>
+          <t>Anthony</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>(502) 554-4833</t>
+          <t>(502) 938-5182</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -525,12 +525,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Autumn</t>
+          <t>Ash</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>(502) 656-2133</t>
+          <t>(502) 554-4833</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -542,12 +542,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Bri</t>
+          <t>Autumn</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>(502) 202-4126</t>
+          <t>(502) 656-2133</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -559,12 +559,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Dakayla</t>
+          <t>Bri</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>(502) 537-8724</t>
+          <t>(502) 202-4126</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -576,12 +576,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Damon</t>
+          <t>Dakayla</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 537-8724</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -593,12 +593,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Divan</t>
+          <t>Damon</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-9406</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -610,12 +610,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Divan</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>(407) 456-1445</t>
+          <t>(502) 821-9406</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -627,12 +627,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>(502) 527-1477</t>
+          <t>(407) 456-1445</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -644,12 +644,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Jada</t>
+          <t>Grace</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-5962</t>
+          <t>(502) 527-1477</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Jeremiah</t>
+          <t>Jada</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>(502) 498-9401</t>
+          <t>(502) 821-5962</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -678,12 +678,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Jeremiah</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(502) 606-3088</t>
+          <t>(502) 498-9401</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -695,12 +695,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Kaisha</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 606-3088</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -712,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Kasey</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(502) 884-2273</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kasey</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 531-8704</t>
+          <t>(502) 884-2273</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 650-2273</t>
+          <t>(502) 531-8704</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 381-0680</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Nyatiek</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(502) 576-1634</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -848,12 +848,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0688</t>
+          <t>(502) 576-1634</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -865,12 +865,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Ryan</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(270) 874-0688</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -882,12 +882,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -899,12 +899,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Vicki</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>(502) 701-9597</t>
+          <t>(502) 724-2384</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -916,22 +916,39 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>(502) 701-9597</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>Zach</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>(502) 422-9066</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C28"/>
+  <autoFilter ref="A1:C29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Daily brief 2026-06-20 — team notes + dashboard wire; directory: remove Damon (failed BG), add Rusul (cleared)
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -593,12 +593,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Damon</t>
+          <t>Divan</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 821-9406</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -610,12 +610,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Divan</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-9406</t>
+          <t>(407) 456-1445</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -627,12 +627,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Grace</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>(407) 456-1445</t>
+          <t>(502) 527-1477</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -644,12 +644,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Jada</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>(502) 527-1477</t>
+          <t>(502) 821-5962</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Jada</t>
+          <t>Jeremiah</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-5962</t>
+          <t>(502) 498-9401</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -678,12 +678,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Jeremiah</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(502) 498-9401</t>
+          <t>(502) 606-3088</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -695,12 +695,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(502) 606-3088</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -712,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Kaisha</t>
+          <t>Kasey</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 884-2273</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kasey</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 884-2273</t>
+          <t>(502) 531-8704</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 531-8704</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 650-2273</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(502) 381-0680</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Nyatiek</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(502) 576-1634</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -848,12 +848,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Nyatiek</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>(502) 576-1634</t>
+          <t>(270) 874-0688</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -865,12 +865,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Rusul</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0688</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily brief 2026-06-26 (rescue) — team notes + dashboard wire; new hire Chloe Hatfield added to directory (29->30)
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -576,12 +576,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Dakayla</t>
+          <t>Chloe</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>(502) 537-8724</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -593,12 +593,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Divan</t>
+          <t>Dakayla</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-9406</t>
+          <t>(502) 537-8724</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -610,12 +610,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Divan</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>(407) 456-1445</t>
+          <t>(502) 821-9406</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -627,12 +627,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>(502) 527-1477</t>
+          <t>(407) 456-1445</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -644,12 +644,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Jada</t>
+          <t>Grace</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-5962</t>
+          <t>(502) 527-1477</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Jeremiah</t>
+          <t>Jada</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>(502) 498-9401</t>
+          <t>(502) 821-5962</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -678,12 +678,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Jeremiah</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(502) 606-3088</t>
+          <t>(502) 498-9401</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -695,12 +695,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Kaisha</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 606-3088</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -712,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Kasey</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(502) 884-2273</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kasey</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 531-8704</t>
+          <t>(502) 884-2273</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 650-2273</t>
+          <t>(502) 531-8704</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 381-0680</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Nyatiek</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(502) 576-1634</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -848,12 +848,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0688</t>
+          <t>(502) 576-1634</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -865,12 +865,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Rusul</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(270) 874-0688</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -882,7 +882,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Ryan Vititoe</t>
+          <t>Rusul</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -899,12 +899,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Ryan Vititoe</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -916,12 +916,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Serina</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 724-2384</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -933,12 +933,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Vicki</t>
+          <t>Serina</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>(502) 701-9597</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -950,22 +950,39 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>(502) 701-9597</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>Zach</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>(502) 422-9066</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C30"/>
+  <autoFilter ref="A1:C31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Daily brief 2026-07-10 — new hire Javeh Goodman added to directory (31->32), team notes + dashboard wire
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -678,12 +678,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Jeremiah</t>
+          <t>Javeh</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(502) 498-9401</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -695,12 +695,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Jeremiah</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(502) 606-3088</t>
+          <t>(502) 498-9401</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -712,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Kaisha</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 606-3088</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kasey</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 884-2273</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kasey</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 531-8704</t>
+          <t>(502) 884-2273</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 650-2273</t>
+          <t>(502) 531-8704</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(502) 381-0680</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Megan</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Megan</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -848,12 +848,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -865,12 +865,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Nyatiek</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>(502) 576-1634</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -882,12 +882,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0688</t>
+          <t>(502) 576-1634</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -899,12 +899,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Rusul</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(270) 874-0688</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -916,7 +916,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Ryan Vititoe</t>
+          <t>Rusul</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -933,12 +933,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Ryan Vititoe</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -950,12 +950,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Serina</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 724-2384</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -967,12 +967,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Vicki</t>
+          <t>Serina</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>(502) 701-9597</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -984,22 +984,39 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>(502) 701-9597</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>Zach</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>(502) 422-9066</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C32"/>
+  <autoFilter ref="A1:C33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
directory: fill new-hire phones — Angela, Javeh, Megan, Rusul, Ryan, Serina
Pulled from BG-check authorization forms (Sent Items, fg2065 mailbox).
Kaisha Brewer remains PHONE PENDING — no BG-check/onboarding email found
in fg2065 for her (established employee, predates the tracked flow).
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 912-4944</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 216-4460</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 833-2695</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 656-9660</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 528-7789</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 777-7987</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">

</xml_diff>

<commit_message>
directory: Kaisha phone (Bobby-provided), add Madelynn Smith new hire
Kaisha Brewer (502) 439-9802 supplied directly by Bobby (no BG-check
email existed for her). Madelynn Haleigh Smith added as new row,
phone (502) 938-3999 pulled from her 6/3 BG-check authorization form
(Sent Items, fg2065 mailbox). 33 rows total.
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -734,7 +734,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 439-9802</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Madelynn</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 938-3999</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Megan</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(502) 833-2695</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -848,12 +848,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Megan</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 833-2695</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -865,12 +865,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -882,12 +882,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Nyatiek</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>(502) 576-1634</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -899,12 +899,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0688</t>
+          <t>(502) 576-1634</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -916,12 +916,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Rusul</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>(502) 656-9660</t>
+          <t>(270) 874-0688</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -933,12 +933,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Ryan Vititoe</t>
+          <t>Rusul</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>(502) 528-7789</t>
+          <t>(502) 656-9660</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -950,12 +950,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Ryan Vititoe</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(502) 528-7789</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -967,12 +967,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Serina</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>(502) 777-7987</t>
+          <t>(502) 724-2384</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -984,12 +984,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Vicki</t>
+          <t>Serina</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>(502) 701-9597</t>
+          <t>(502) 777-7987</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1001,22 +1001,39 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>(502) 701-9597</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t>Zach</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>(502) 422-9066</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C33"/>
+  <autoFilter ref="A1:C34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
directory: add Cortez Brown (new hire, cleared 2026-08-07); refresh shop performance + daily missing temps
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -593,12 +593,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Dakayla</t>
+          <t>Cortez</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>(502) 537-8724</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -610,12 +610,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Divan</t>
+          <t>Dakayla</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-9406</t>
+          <t>(502) 537-8724</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -627,12 +627,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Divan</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>(407) 456-1445</t>
+          <t>(502) 821-9406</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -644,12 +644,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>(502) 527-1477</t>
+          <t>(407) 456-1445</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Jada</t>
+          <t>Grace</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-5962</t>
+          <t>(502) 527-1477</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -678,12 +678,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Javeh</t>
+          <t>Jada</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(502) 216-4460</t>
+          <t>(502) 821-5962</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -695,12 +695,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Jeremiah</t>
+          <t>Javeh</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(502) 498-9401</t>
+          <t>(502) 216-4460</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -712,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Jeremiah</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(502) 606-3088</t>
+          <t>(502) 498-9401</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kaisha</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 439-9802</t>
+          <t>(502) 606-3088</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kasey</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 884-2273</t>
+          <t>(502) 439-9802</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kasey</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 531-8704</t>
+          <t>(502) 884-2273</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(502) 650-2273</t>
+          <t>(502) 531-8704</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(502) 381-0680</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Madelynn</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(502) 938-3999</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Madelynn</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 938-3999</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -848,12 +848,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Megan</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>(502) 833-2695</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -865,12 +865,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Megan</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 833-2695</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -882,12 +882,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -899,12 +899,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Nyatiek</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>(502) 576-1634</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -916,12 +916,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0688</t>
+          <t>(502) 576-1634</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -933,12 +933,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Rusul</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>(502) 656-9660</t>
+          <t>(270) 874-0688</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -950,12 +950,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Ryan Vititoe</t>
+          <t>Rusul</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>(502) 528-7789</t>
+          <t>(502) 656-9660</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -967,12 +967,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Ryan Vititoe</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(502) 528-7789</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -984,12 +984,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Serina</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>(502) 777-7987</t>
+          <t>(502) 724-2384</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1001,12 +1001,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Vicki</t>
+          <t>Serina</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>(502) 701-9597</t>
+          <t>(502) 777-7987</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1018,22 +1018,39 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>(502) 701-9597</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>Zach</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>(502) 422-9066</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C34"/>
+  <autoFilter ref="A1:C35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>